<commit_message>
Added TestScript31 ,TestScript32 and updated excel file
</commit_message>
<xml_diff>
--- a/data/TestData.xlsx
+++ b/data/TestData.xlsx
@@ -4,15 +4,14 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9302"/>
   <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="20115" windowHeight="7500"/>
+    <workbookView xWindow="0" yWindow="2445" windowWidth="21570" windowHeight="11175"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
-    <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
-    <sheet name="TestCase" r:id="rId7" sheetId="4"/>
+    <sheet name="Multiple" sheetId="1" r:id="rId1"/>
+    <sheet name="TestCase" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="145621"/>
+  <calcPr calcId="0"/>
+  <oleSize ref="A1:T35"/>
 </workbook>
 </file>
 
@@ -50,7 +49,6 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <numFmts count="0"/>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -397,20 +395,20 @@
   <dimension ref="A1:B4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="12.7109375"/>
-    <col min="2" max="2" customWidth="true" width="18.42578125"/>
+    <col min="1" max="1" width="12.7109375" customWidth="1"/>
+    <col min="2" max="2" width="18.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" t="s" s="0">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s" s="0">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" t="s" s="0">
+      <c r="A2" t="s">
         <v>2</v>
       </c>
       <c r="B2" s="1" t="s">
@@ -418,7 +416,7 @@
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" t="s" s="0">
+      <c r="A3" t="s">
         <v>7</v>
       </c>
       <c r="B3" s="1" t="s">
@@ -426,7 +424,7 @@
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" t="s" s="0">
+      <c r="A4" t="s">
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
@@ -447,31 +445,13 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15.0"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="s" s="0">
-        <v>8</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
yet to compelte -Pending
</commit_message>
<xml_diff>
--- a/data/TestData.xlsx
+++ b/data/TestData.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
   <si>
     <t xml:space="preserve">Name </t>
   </si>
@@ -43,6 +43,24 @@
   </si>
   <si>
     <t>Hello</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC ID </t>
+  </si>
+  <si>
+    <t>Rama</t>
+  </si>
+  <si>
+    <t>Shyam</t>
+  </si>
+  <si>
+    <t>Rama@gmail.com</t>
+  </si>
+  <si>
+    <t>Shyam@gmail.com</t>
+  </si>
+  <si>
+    <t>TC Status</t>
   </si>
 </sst>
 </file>
@@ -87,9 +105,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" quotePrefix="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -392,43 +412,80 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
     <col min="2" max="2" width="18.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>2</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C2">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>7</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C3">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>6</v>
+      </c>
+      <c r="C4">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C5">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C6">
+        <v>105</v>
       </c>
     </row>
   </sheetData>
@@ -436,6 +493,8 @@
     <hyperlink ref="B2" r:id="rId1"/>
     <hyperlink ref="B3" r:id="rId2"/>
     <hyperlink ref="B4" r:id="rId3"/>
+    <hyperlink ref="B5" r:id="rId4"/>
+    <hyperlink ref="B6" r:id="rId5"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Updated creatAdminData() with generic excel methods
</commit_message>
<xml_diff>
--- a/data/TestData.xlsx
+++ b/data/TestData.xlsx
@@ -29,81 +29,64 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t xml:space="preserve">Name </t>
   </si>
   <si>
-    <t>Email ID</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TC ID </t>
-  </si>
-  <si>
-    <t>TC Status</t>
-  </si>
-  <si>
-    <t>Jhon</t>
-  </si>
-  <si>
-    <t>Jhon@gmail.com</t>
-  </si>
-  <si>
-    <t>101</t>
-  </si>
-  <si>
-    <t>Pass</t>
-  </si>
-  <si>
     <t>smith</t>
   </si>
   <si>
     <t>smith@gmail.com</t>
   </si>
   <si>
-    <t>102</t>
-  </si>
-  <si>
     <t>admin</t>
   </si>
   <si>
     <t>admin@gmail.com</t>
   </si>
   <si>
-    <t>103</t>
-  </si>
-  <si>
     <t>Rama</t>
   </si>
   <si>
     <t>Rama@gmail.com</t>
   </si>
   <si>
-    <t>104</t>
-  </si>
-  <si>
     <t>Shyam</t>
   </si>
   <si>
     <t>Shyam@gmail.com</t>
   </si>
   <si>
-    <t>105</t>
-  </si>
-  <si>
     <t>Hello</t>
+  </si>
+  <si>
+    <t>password</t>
+  </si>
+  <si>
+    <t>Ravi123</t>
+  </si>
+  <si>
+    <t>Ravi M B</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -148,7 +131,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -158,6 +141,9 @@
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -465,7 +451,7 @@
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
-    <col min="2" max="2" width="18.42578125" customWidth="1"/>
+    <col min="2" max="2" width="19.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -473,99 +459,63 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
+        <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="E2" s="3"/>
+      <c r="A2" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2" s="3"/>
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="4" t="s">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="E3" s="3"/>
+        <v>2</v>
+      </c>
+      <c r="C3" s="3"/>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="4" t="s">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="E4" s="3"/>
+        <v>4</v>
+      </c>
+      <c r="C4" s="3"/>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" s="4" t="s">
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="E5" s="3"/>
+        <v>6</v>
+      </c>
+      <c r="C5" s="3"/>
     </row>
     <row r="6" spans="1:5">
       <c r="A6" s="4" t="s">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="E6" s="3"/>
+        <v>8</v>
+      </c>
+      <c r="C6" s="3"/>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B2" r:id="rId1"/>
-    <hyperlink ref="B3" r:id="rId2"/>
-    <hyperlink ref="B4" r:id="rId3"/>
-    <hyperlink ref="B5" r:id="rId4"/>
-    <hyperlink ref="B6" r:id="rId5"/>
+    <hyperlink ref="B3" r:id="rId1"/>
+    <hyperlink ref="B4" r:id="rId2"/>
+    <hyperlink ref="B5" r:id="rId3"/>
+    <hyperlink ref="B6" r:id="rId4"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId5"/>
 </worksheet>
 </file>
 
@@ -576,7 +526,7 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" t="s">
-        <v>20</v>
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added verify titile Test method
</commit_message>
<xml_diff>
--- a/data/TestData.xlsx
+++ b/data/TestData.xlsx
@@ -7,7 +7,7 @@
     <workbookView xWindow="0" yWindow="2445" windowWidth="21510" windowHeight="11175"/>
   </bookViews>
   <sheets>
-    <sheet name="EMPDATA" sheetId="1" r:id="rId1"/>
+    <sheet name="Login" sheetId="1" r:id="rId1"/>
     <sheet name="TestCase" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
@@ -64,10 +64,10 @@
     <t>password</t>
   </si>
   <si>
-    <t>Ravi123</t>
-  </si>
-  <si>
-    <t>Ravi M B</t>
+    <t>Admin</t>
+  </si>
+  <si>
+    <t>admin123</t>
   </si>
 </sst>
 </file>
@@ -464,10 +464,10 @@
     </row>
     <row r="2" spans="1:5">
       <c r="A2" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B2" s="5" t="s">
         <v>12</v>
-      </c>
-      <c r="B2" s="5" t="s">
-        <v>11</v>
       </c>
       <c r="C2" s="3"/>
     </row>

</xml_diff>